<commit_message>
Add full sourcing: classify every figure (Reported/Derived/Estimate)
- New 'Sources & Methodology' tab documenting source + URL for every figure,
  with EBITDA estimate basis (group D&A ~7.7% of sales; segment add-backs 3.75%/2.75%)
- Add 'Mult. basis' + 'Source ref' columns to both comp tabs; n/d values excluded
  from medians/means
- Correct Nestle/Gerber EBITDA multiple to 15.7x FY07e (Washington Post) from prior ~20x estimate
- Sync markdown report and comps CSV with the same basis flags
</commit_message>
<xml_diff>
--- a/abbott-precedent-transaction-analysis/Abbott_Nutrition_and_EPD_Precedent_Transaction_Analysis.xlsx
+++ b/abbott-precedent-transaction-analysis/Abbott_Nutrition_and_EPD_Precedent_Transaction_Analysis.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Nutrition Comps" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="EPD Comps" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Valuation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sources &amp; Methodology" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="#,##0.0&quot;bn&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +72,12 @@
     <font>
       <name val="Calibri"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="8">
@@ -137,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -267,6 +274,15 @@
     </xf>
     <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -352,7 +368,7 @@
   <commentList>
     <comment ref="A12" authorId="0" shapeId="0">
       <text>
-        <t>Abbott does not publish EBITDA by segment. Estimated by adding assumed D&amp;A to disclosed segment operating earnings.</t>
+        <t>ESTIMATE. Abbott does not publish EBITDA by segment. = disclosed segment operating earnings + assumed D&amp;A add-back. See Sources tab note S4.</t>
       </text>
     </comment>
   </commentList>
@@ -651,7 +667,7 @@
   <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -669,14 +685,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Potential divestiture of the Nutrition and Established Pharmaceuticals (EPD) businesses  •  FY2024 basis  •  Indicative / discussion draft</t>
+          <t>Potential divestiture of Nutrition and Established Pharmaceuticals (EPD)  •  FY2024 basis  •  Indicative / discussion draft</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Headline indicative enterprise value (EV) — see Valuation tab for build, Inputs tab for assumptions.</t>
+          <t>Headline indicative EV. Build = Valuation tab; assumptions = Inputs tab; every figure sourced/flagged on Sources &amp; Methodology tab.</t>
         </is>
       </c>
     </row>
@@ -727,15 +743,15 @@
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>TEXT('Inputs &amp; Assumptions'!B17,"0.0")&amp;"–"&amp;TEXT('Inputs &amp; Assumptions'!C17,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!B17,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!C17,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>TEXT('Inputs &amp; Assumptions'!B18,"0.0")&amp;"–"&amp;TEXT('Inputs &amp; Assumptions'!C18,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!B18,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!C18,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="F7" s="8">
-        <f>TEXT(Valuation!D8/1000,"0")&amp;"–"&amp;TEXT(Valuation!E8/1000,"0")&amp;"bn"</f>
+        <f>TEXT(Valuation!D8/1000,"0")&amp;"-"&amp;TEXT(Valuation!E8/1000,"0")&amp;"bn"</f>
         <v/>
       </c>
     </row>
@@ -754,15 +770,15 @@
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>TEXT('Inputs &amp; Assumptions'!D17,"0.0")&amp;"–"&amp;TEXT('Inputs &amp; Assumptions'!E17,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!D17,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!E17,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>TEXT('Inputs &amp; Assumptions'!D18,"0.0")&amp;"–"&amp;TEXT('Inputs &amp; Assumptions'!E18,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!D18,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!E18,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>TEXT(Valuation!D14/1000,"0")&amp;"–"&amp;TEXT(Valuation!E14/1000,"0")&amp;"bn"</f>
+        <f>TEXT(Valuation!D14/1000,"0")&amp;"-"&amp;TEXT(Valuation!E14/1000,"0")&amp;"bn"</f>
         <v/>
       </c>
     </row>
@@ -791,7 +807,7 @@
         </is>
       </c>
       <c r="F9" s="16">
-        <f>TEXT((Valuation!D8+Valuation!D14)/1000,"0")&amp;"–"&amp;TEXT((Valuation!E8+Valuation!E14)/1000,"0")&amp;"bn"</f>
+        <f>TEXT((Valuation!D8+Valuation!D14)/1000,"0")&amp;"-"&amp;TEXT((Valuation!E8+Valuation!E14)/1000,"0")&amp;"bn"</f>
         <v/>
       </c>
     </row>
@@ -805,42 +821,42 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>•  EPD is the cleaner asset — high-growth (+9.2%), high-margin (23.7%) emerging-market branded generics; sits at the premium end of the branded-generics deal range.</t>
+          <t>•  EPD: high-growth (+9.2%), high-margin (23.7%) EM branded generics — premium end of the branded-generics deal range.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>•  Nutrition is two-speed: attractive, growing adult/medical nutrition (Ensure, Glucerna) vs. a structurally challenged infant-formula half (Similac) carrying an NEC product-liability litigation overhang.</t>
+          <t>•  Nutrition: two-speed — growing adult/medical nutrition (Ensure, Glucerna) vs. structurally challenged infant formula (Similac) with an NEC litigation overhang [S19].</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>•  Peak infant-formula comps (Reckitt/MJN 17.4x, Nestlé/Pfizer ~20x) are discounted for Nutrition's blended mix and litigation risk.</t>
+          <t>•  Peak infant-formula comps (Reckitt/MJN 17.4x; Nestlé/Pfizer ~20-24x) discounted for Nutrition's blend and litigation risk.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>•  Sum-of-the-parts optionality: selling adult nutrition at consumer-health multiples while ring-fencing infant formula could exceed the blended range.</t>
+          <t>•  Sum-of-the-parts optionality: adult nutrition at consumer-health multiples while ring-fencing infant formula could exceed the blended range.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>•  EBITDA is ESTIMATED (Abbott discloses segment operating margin, not EBITDA). Indicative only — not investment advice; refine with carve-out QoE financials.</t>
+          <t>•  EBITDA is ESTIMATED (Abbott discloses segment margin, not EBITDA). Every figure's basis is on the Sources &amp; Methodology tab.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Tabs:  Summary  ·  Inputs &amp; Assumptions (drivers)  ·  Nutrition Comps  ·  EPD Comps  ·  Valuation (build)</t>
+          <t>Tabs:  Summary  ·  Inputs &amp; Assumptions  ·  Nutrition Comps  ·  EPD Comps  ·  Valuation  ·  Sources &amp; Methodology</t>
         </is>
       </c>
     </row>
@@ -867,12 +883,10 @@
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -885,14 +899,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Blue cells are inputs — change them and the Valuation/Summary tabs recalc. FY2024 reported segment basis. EBITDA is estimated (see notes).</t>
+          <t>Blue = input cells (change to recalc). FY2024 reported basis. EBITDA is ESTIMATED — see 'Sources &amp; Methodology' tab for the basis of every figure.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Blue figures are drivers. $ figures in US$ millions unless noted.</t>
+          <t>Blue figures are drivers. $ figures in US$ millions unless noted. Ref column shows source/estimate basis (full detail on Sources tab).</t>
         </is>
       </c>
     </row>
@@ -921,7 +935,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Source / note</t>
+          <t>Basis / source (see Sources tab)</t>
         </is>
       </c>
     </row>
@@ -939,7 +953,7 @@
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Abbott FY24 segment reporting (~$8.4bn / ~$5.2bn)</t>
+          <t>REPORTED — Abbott FY24 segment reporting [S1, S2]</t>
         </is>
       </c>
     </row>
@@ -957,7 +971,7 @@
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>Disclosed: Nutrition 17.9%, EPD 23.7%</t>
+          <t>REPORTED — Abbott (Nutrition 17.9%, EPD 23.7%) [S3]</t>
         </is>
       </c>
     </row>
@@ -975,7 +989,7 @@
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Estimate — Nutrition more capital-intensive</t>
+          <t>ESTIMATE — benchmarked to group D&amp;A ~7.7% of sales (amort. concentrated in MedDev/Dx) [S4]</t>
         </is>
       </c>
     </row>
@@ -993,9 +1007,10 @@
         <f>C8*C9</f>
         <v/>
       </c>
-      <c r="D11" s="23">
-        <f> sales x operating margin</f>
-        <v/>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>DERIVED = sales x operating margin</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1012,9 +1027,10 @@
         <f>C8*(C9+C10)</f>
         <v/>
       </c>
-      <c r="D12" s="26">
-        <f> operating earnings + D&amp;A add-back</f>
-        <v/>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>ESTIMATE = operating earnings + D&amp;A add-back</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1031,12 +1047,16 @@
         <f>C12/C8</f>
         <v/>
       </c>
-      <c r="D13" s="27" t="inlineStr"/>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>Selected multiple ranges (judgement)</t>
+          <t>Selected multiple ranges (judgement — see rationale below)</t>
         </is>
       </c>
     </row>
@@ -1108,28 +1128,28 @@
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>Rationale</t>
+          <t>Rationale for selected ranges</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="18" t="inlineStr">
         <is>
-          <t>•  Nutrition: peak infant-formula comps (Reckitt/MJN 17.4x, Nestlé/Pfizer ~20x) discounted for blended adult+pediatric mix and the NEC litigation overhang.</t>
+          <t>•  Nutrition: peak infant-formula comps (Reckitt/MJN 17.4x, Nestlé/Pfizer ~20-24x) DISCOUNTED for blended adult+pediatric mix and the NEC litigation overhang [S5].</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t>•  EPD: premium end of branded-generics range (STADA 13.4x / Krka ~11.5x) given +9.2% growth and 23.7% margin; above mature Western generics (Hikma/Richter ~6x).</t>
+          <t>•  EPD: premium end of branded-generics range (STADA 13.4x / 11.3x; Krka ~11.5x) given +9.2% growth and 23.7% margin; above mature Western generics (Hikma/Richter ~6x) [S6].</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t>•  EBITDA is ESTIMATED — Abbott discloses segment operating margin, not EBITDA. Refine with carve-out quality-of-earnings financials.</t>
+          <t>•  EBITDA is ESTIMATED — Abbott discloses segment operating margin, not segment EBITDA. Refine with carve-out quality-of-earnings financials [S4].</t>
         </is>
       </c>
     </row>
@@ -1152,16 +1172,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1174,7 +1196,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Precedent transactions — infant + adult/medical nutrition. Multiples as reported by public sources; treat as directional.</t>
+          <t>Precedent transactions — infant + adult/medical nutrition. 'Mult. basis' flags Reported vs Derived vs estimate. Full citations on Sources tab.</t>
         </is>
       </c>
     </row>
@@ -1210,6 +1232,16 @@
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Mult. basis</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Source ref</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1233,12 +1265,22 @@
         <v>16.8</v>
       </c>
       <c r="E5" s="30" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="F5" s="30" t="n">
         <v>22</v>
       </c>
       <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>EV/S derived (÷FY06 sales €2.6bn); EBITDA per press</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
         <is>
           <t>Baby + medical nutrition; peak strategic multiple</t>
         </is>
@@ -1255,7 +1297,7 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Gerber (from Novartis)</t>
+          <t>Gerber (Novartis)</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
@@ -1265,11 +1307,21 @@
         <v>2.8</v>
       </c>
       <c r="F6" s="32" t="n">
-        <v>20</v>
+        <v>15.7</v>
       </c>
       <c r="G6" s="31" t="inlineStr">
         <is>
-          <t>EBITDA mult. est.; made Nestlé #1 baby food</t>
+          <t>EV/S derived; EBITDA reported (15.7x FY07e)</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="I6" s="31" t="inlineStr">
+        <is>
+          <t>Made Nestlé #1 in baby food</t>
         </is>
       </c>
     </row>
@@ -1294,11 +1346,21 @@
         <v>5</v>
       </c>
       <c r="F7" s="30" t="n">
-        <v>22</v>
+        <v>23.7</v>
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>~$2.1bn sales / ~$0.5bn EBITDA (2011); EM (China) entry</t>
+          <t>EV/S derived (4.9x FY12e / 5.6x FY11); EBITDA derived ($0.5bn '11); press ~20x fwd</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>EM (China) entry</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1389,17 @@
       </c>
       <c r="G8" s="31" t="inlineStr">
         <is>
-          <t>Organic/plant-based (not infant); lower-multiple bookend</t>
+          <t>EV/S reported (FY17); EBITDA reported (~19.8-20x FY16e)</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="I8" s="31" t="inlineStr">
+        <is>
+          <t>Organic/plant-based; lower-multiple bookend (not infant)</t>
         </is>
       </c>
     </row>
@@ -1356,6 +1428,16 @@
       </c>
       <c r="G9" s="20" t="inlineStr">
         <is>
+          <t>EV/S reported (FY15); EBITDA reported (FY16)</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
           <t>Pure-play infant formula; closest single comp (~14x w/ synergies)</t>
         </is>
       </c>
@@ -1378,12 +1460,24 @@
         <v>5.75</v>
       </c>
       <c r="E10" s="32" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="F10" s="32" t="n">
-        <v>17</v>
+        <v>2.9</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
       </c>
       <c r="G10" s="31" t="inlineStr">
+        <is>
+          <t>EV/S derived (÷~$2.0bn sales); EBITDA n/d</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="I10" s="31" t="inlineStr">
         <is>
           <t>Vitamins/supplements; adult-nutrition-adjacent</t>
         </is>
@@ -1410,6 +1504,8 @@
         <v/>
       </c>
       <c r="G11" s="34" t="inlineStr"/>
+      <c r="H11" s="34" t="inlineStr"/>
+      <c r="I11" s="34" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="33" t="inlineStr">
@@ -1432,11 +1528,21 @@
         <v/>
       </c>
       <c r="G12" s="34" t="inlineStr"/>
+      <c r="H12" s="34" t="inlineStr"/>
+      <c r="I12" s="34" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>n/d = not disclosed / not reliably sourced (excluded from median &amp; mean).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1448,16 +1554,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1470,7 +1578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Precedent transactions — branded / emerging-market generics. Listed reads for context: Krka ~11.5x, Hikma ~6.3x, Richter ~6x EV/EBITDA.</t>
+          <t>Precedent transactions — branded / EM generics. Listed reads for context: Krka ~11.5x, Hikma ~6.3x, Richter ~6x EV/EBITDA [S6].</t>
         </is>
       </c>
     </row>
@@ -1506,6 +1614,16 @@
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Mult. basis</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Source ref</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1531,10 +1649,24 @@
       <c r="E5" s="30" t="n">
         <v>2.2</v>
       </c>
-      <c r="F5" s="30" t="n"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
       <c r="G5" s="20" t="inlineStr">
         <is>
-          <t>Incl. debt; low-margin target (EBITDA mult. n/m); India/EM</t>
+          <t>EV/S derived (÷~$1.8bn sales); EBITDA n/d (low margin)</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>India/EM generics consolidation</t>
         </is>
       </c>
     </row>
@@ -1555,15 +1687,29 @@
       <c r="D6" s="10" t="n">
         <v>40.5</v>
       </c>
-      <c r="E6" s="32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="F6" s="32" t="n">
-        <v>11.5</v>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
       </c>
       <c r="G6" s="31" t="inlineStr">
         <is>
-          <t>EBITDA mult. est.; global generics scale</t>
+          <t>EV reported; multiples n/d (analyst ~12-13x w/ synergies)</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="I6" s="31" t="inlineStr">
+        <is>
+          <t>Global generics scale; widely viewed as full price</t>
         </is>
       </c>
     </row>
@@ -1585,14 +1731,24 @@
         <v>9.9</v>
       </c>
       <c r="E7" s="30" t="n">
-        <v>3.3</v>
+        <v>4</v>
       </c>
       <c r="F7" s="30" t="n">
         <v>10.5</v>
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>8.9x w/ synergies; ~10–11x reported; branded/specialty + EM/OTC</t>
+          <t>EV/S derived (~4x FY15 sales); EBITDA reported (8.9x w/ syn; ~10-11x rep.)</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>Branded/specialty + EM/OTC reach</t>
         </is>
       </c>
     </row>
@@ -1614,14 +1770,24 @@
         <v>5.7</v>
       </c>
       <c r="E8" s="32" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="F8" s="32" t="n">
         <v>13.4</v>
       </c>
       <c r="G8" s="31" t="inlineStr">
         <is>
-          <t>EUR 5.32bn; PE take-private; branded generics + consumer health</t>
+          <t>EV/S derived (÷FY16 sales €2.14bn); EBITDA reported (FY16)</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="I8" s="31" t="inlineStr">
+        <is>
+          <t>PE take-private; branded generics + consumer health</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1816,17 @@
       </c>
       <c r="G9" s="20" t="inlineStr">
         <is>
-          <t>EUR ~1.9bn; EU/EM branded-generics carve-out</t>
+          <t>EV/S derived (approx); EBITDA reported (10.25x)</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>EU/EM branded-generics carve-out</t>
         </is>
       </c>
     </row>
@@ -1672,14 +1848,24 @@
         <v>10</v>
       </c>
       <c r="E10" s="32" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="F10" s="32" t="n">
         <v>11.3</v>
       </c>
       <c r="G10" s="31" t="inlineStr">
         <is>
-          <t>Reported ~EUR 10bn; latest large branded-generics print</t>
+          <t>EV/S derived (÷FY24 sales ~€4.1bn); EBITDA reported (11.29x)</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="I10" s="31" t="inlineStr">
+        <is>
+          <t>Latest large branded-generics print; re-rate vs 2017</t>
         </is>
       </c>
     </row>
@@ -1704,6 +1890,8 @@
         <v/>
       </c>
       <c r="G11" s="34" t="inlineStr"/>
+      <c r="H11" s="34" t="inlineStr"/>
+      <c r="I11" s="34" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="33" t="inlineStr">
@@ -1726,11 +1914,21 @@
         <v/>
       </c>
       <c r="G12" s="34" t="inlineStr"/>
+      <c r="H12" s="34" t="inlineStr"/>
+      <c r="I12" s="34" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>n/d = not disclosed / not reliably sourced (excluded from median &amp; mean).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1763,7 +1961,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Driven by Inputs &amp; Assumptions tab. $ in US$ millions; EV summary in $bn.</t>
+          <t>Driven by Inputs &amp; Assumptions tab. $ in US$m; EV midpoint shown in $bn.</t>
         </is>
       </c>
     </row>
@@ -2050,4 +2248,704 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sources &amp; Methodology</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Every figure classified REPORTED (from a primary/press source), DERIVED (calculated), or ESTIMATE (analyst judgement). Click links to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>A. Target financials &amp; EBITDA estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Item / figure</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Value used</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Abbott total net sales FY2024</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>$41,950m</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E6" s="44" t="inlineStr">
+        <is>
+          <t>Abbott FY2024 Form 10-K (FY ended 31-Dec-2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Nutrition ~$8.41bn; EPD ~$5.19bn; Dx ~$9.34bn FY24 segment sales</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>$8.41bn / $5.19bn</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E7" s="44" t="inlineStr">
+        <is>
+          <t>Abbott segment reporting (Bullfincher; Statista)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Segment operating margin: Nutrition 17.9%, EPD 23.7%; growth +5.9% / +9.2%</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>17.9% / 23.7%</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E8" s="44" t="inlineStr">
+        <is>
+          <t>Abbott FY2024 10-K MD&amp;A (segment results)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Group D&amp;A FY24: Depreciation ~$1,340m + Amort. of intangibles ~$1,878m = ~$3,218m (~7.7% of sales). Amortization concentrated in Med Devices/Diagnostics (acquired intangibles), so Nutrition/EPD add-backs (depreciation-led) assumed below group: 3.75% / 2.75% of sales.</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>D&amp;A add-back 3.75% / 2.75%</t>
+        </is>
+      </c>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E9" s="44" t="inlineStr">
+        <is>
+          <t>Abbott FY2024 cash-flow disclosure (per 10-Q/10-K); segment split is analyst judgement</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Implied segment operating earnings (Nutrition ~$1.50bn; EPD ~$1.23bn)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>sales x margin</t>
+        </is>
+      </c>
+      <c r="D10" s="46" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Calculation (S2 x S3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Estimated segment EBITDA: Nutrition ~$1.7-1.9bn; EPD ~$1.3-1.45bn</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>op earnings + D&amp;A</t>
+        </is>
+      </c>
+      <c r="D11" s="45" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>Calculation (operating earnings + S4 add-back)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>B. Precedent transaction sources (multiples)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Transaction</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Key reported figure</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Comp discount rationale (Nutrition)</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>Peak comps discounted</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>Analyst judgement — see Nutrition Comps &amp; RB/MJN coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Listed branded-generics reads: Krka ~11.5x, Hikma ~6.3x, Richter ~6x; Zentiva 10.25x, STADA 11.29x</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>Context multiples</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E16" s="44" t="inlineStr">
+        <is>
+          <t>InterCapital — European pharma generics M&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>Danone / Numico (2007)</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>€12.3bn EV; ~22x EBITDA; FY06 sales €2.6bn (18.4% EBITA margin)</t>
+        </is>
+      </c>
+      <c r="D17" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E17" s="44" t="inlineStr">
+        <is>
+          <t>Danone analyst presentation (Jul-2007); 22x cited in RB/MJN coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Nestlé / Gerber (2007)</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>$5.5bn EV; 15.7x FY07e EBITDA; FY07e sales $1.95bn</t>
+        </is>
+      </c>
+      <c r="D18" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="inlineStr">
+        <is>
+          <t>Washington Post (Apr-2007); Nestlé/Novartis releases</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Nestlé / Pfizer Nutrition (2012)</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>$11.85bn EV; FY11 sales $2.1bn, EBITDA $0.5bn (=23.7x); press ~20x fwd</t>
+        </is>
+      </c>
+      <c r="D19" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E19" s="44" t="inlineStr">
+        <is>
+          <t>Proactive Investors; Pfizer 8-K (SEC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Danone / WhiteWave (2016/17)</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>$12.5bn EV; 2.7x FY17 sales; ~19.8-20x FY16e EBITDA</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E20" s="44" t="inlineStr">
+        <is>
+          <t>FoodNavigator-USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>Reckitt / Mead Johnson (2017)</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>$17.9bn EV; 4.4x FY15 sales; 17.4x FY16 EBITDA (~14x w/ syn.)</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E21" s="44" t="inlineStr">
+        <is>
+          <t>Bocconi BSIC; Mead Johnson 8-K (SEC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Nestlé / The Bountiful Company (2021)</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>$5.75bn EV; ~$2.0bn sales (=~2.9x); EBITDA n/d</t>
+        </is>
+      </c>
+      <c r="D22" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>Nestlé press (Aug-2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>Sun Pharma / Ranbaxy (2014)</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>~$4.0bn EV incl. debt; ~$1.8bn sales (=~2.2x); EBITDA n/d</t>
+        </is>
+      </c>
+      <c r="D23" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>Sun Pharma / Ranbaxy deal disclosures</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Teva / Allergan Generics (Actavis, 2015)</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>$40.5bn EV (closed ~$39.5bn); multiples n/d (analyst ~12-13x)</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E24" s="44" t="inlineStr">
+        <is>
+          <t>SEC Form 425 (Allergan); analyst commentary</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>Mylan / Meda (2016)</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>$9.9bn EV; 8.9x adj. EBITDA w/ synergies; FY15 sales ~$2.3bn (=~4.0x)</t>
+        </is>
+      </c>
+      <c r="D25" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E25" s="44" t="inlineStr">
+        <is>
+          <t>Mylan 8-K (SEC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Bain/Cinven / STADA (2017)</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>€5.32bn EV; 13.4x FY16 EBITDA; FY16 sales €2.14bn (=~2.5x)</t>
+        </is>
+      </c>
+      <c r="D26" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E26" s="44" t="inlineStr">
+        <is>
+          <t>Bocconi BSIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>Advent / Zentiva (2018)</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>~€1.9bn EV; ~10.25x EBITDA; ~2.5x sales</t>
+        </is>
+      </c>
+      <c r="D27" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E27" s="44" t="inlineStr">
+        <is>
+          <t>InterCapital</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>CapVest / STADA majority (2025)</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>~€10bn EV reported; ~11.29x EBITDA; FY24 sales ~€4.1bn (=~2.4x)</t>
+        </is>
+      </c>
+      <c r="D28" s="46" t="inlineStr">
+        <is>
+          <t>REPORTED/DERIVED</t>
+        </is>
+      </c>
+      <c r="E28" s="44" t="inlineStr">
+        <is>
+          <t>Bain Capital/Cinven press; InterCapital</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="inlineStr">
+        <is>
+          <t>NEC infant-formula litigation overhang</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>$495m (2024), $58-60m (2025-26) verdicts; ~683 active cases (Apr-25)</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>REPORTED</t>
+        </is>
+      </c>
+      <c r="E29" s="44" t="inlineStr">
+        <is>
+          <t>Reuters/Yahoo; Top Class Actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Legend:  REPORTED = from a primary filing or press source  ·  DERIVED = calculated (EV ÷ sales/EBITDA)  ·  ESTIMATE = analyst judgement.  Multiples across sources may use different EBITDA definitions / years; treat as directional. Not investment advice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A31:E31"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId16"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add carve-out standalone/dis-synergy + NEC assumptions and Sensitivity tab
- Inputs tab: standalone cost (1.5% Nutrition / 2.0% EPD of sales) -> standalone-
  adjusted EBITDA drives EV/EBITDA; illustrative $1.5bn NEC risk deduction netted
  off Nutrition EV; all editable
- Valuation tab: EV/EBITDA now on standalone EBITDA; Nutrition shows pre-litigation
  blended -> less NEC -> adjusted EV; combined uses adjusted Nutrition
- New Sensitivity tab: two live 2-way tables (EV/EBITDA x standalone cost; NEC x cost)
- Sources tab: S20 (standalone cost), S21 (NEC deduction), S22 (stranded costs) basis
- Markdown report: new section 6.5 (carve-out/standalone/stranded assumptions),
  updated headline (post-adjustment combined ~$28-42bn vs pre-adjustment ~$31-45bn)
- Stranded costs flagged as RemainCo (seller-side), not deducted from target EV
</commit_message>
<xml_diff>
--- a/abbott-precedent-transaction-analysis/Abbott_Nutrition_and_EPD_Precedent_Transaction_Analysis.xlsx
+++ b/abbott-precedent-transaction-analysis/Abbott_Nutrition_and_EPD_Precedent_Transaction_Analysis.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Nutrition Comps" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="EPD Comps" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Valuation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sources &amp; Methodology" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sensitivity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sources &amp; Methodology" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -144,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -274,6 +275,18 @@
     </xf>
     <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -664,12 +677,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -709,7 +722,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Est. EBITDA ($bn)</t>
+          <t>Standalone EBITDA ($bn)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -739,19 +752,19 @@
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>'Inputs &amp; Assumptions'!B12/1000</f>
+        <f>'Inputs &amp; Assumptions'!B18/1000</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>TEXT('Inputs &amp; Assumptions'!B17,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!C17,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!B23,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!C23,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>TEXT('Inputs &amp; Assumptions'!B18,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!C18,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!B24,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!C24,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="F7" s="8">
-        <f>TEXT(Valuation!D8/1000,"0")&amp;"-"&amp;TEXT(Valuation!E8/1000,"0")&amp;"bn"</f>
+        <f>TEXT(Valuation!D10/1000,"0")&amp;"-"&amp;TEXT(Valuation!E10/1000,"0")&amp;"bn"</f>
         <v/>
       </c>
     </row>
@@ -766,19 +779,19 @@
         <v/>
       </c>
       <c r="C8" s="10">
-        <f>'Inputs &amp; Assumptions'!C12/1000</f>
+        <f>'Inputs &amp; Assumptions'!C18/1000</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>TEXT('Inputs &amp; Assumptions'!D17,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!E17,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!D23,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!E23,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>TEXT('Inputs &amp; Assumptions'!D18,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!E18,"0.0")&amp;"x"</f>
+        <f>TEXT('Inputs &amp; Assumptions'!D24,"0.0")&amp;"-"&amp;TEXT('Inputs &amp; Assumptions'!E24,"0.0")&amp;"x"</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>TEXT(Valuation!D14/1000,"0")&amp;"-"&amp;TEXT(Valuation!E14/1000,"0")&amp;"bn"</f>
+        <f>TEXT(Valuation!D16/1000,"0")&amp;"-"&amp;TEXT(Valuation!E16/1000,"0")&amp;"bn"</f>
         <v/>
       </c>
     </row>
@@ -793,7 +806,7 @@
         <v/>
       </c>
       <c r="C9" s="14">
-        <f>('Inputs &amp; Assumptions'!B12+'Inputs &amp; Assumptions'!C12)/1000</f>
+        <f>('Inputs &amp; Assumptions'!B18+'Inputs &amp; Assumptions'!C18)/1000</f>
         <v/>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -807,7 +820,7 @@
         </is>
       </c>
       <c r="F9" s="16">
-        <f>TEXT((Valuation!D8+Valuation!D14)/1000,"0")&amp;"-"&amp;TEXT((Valuation!E8+Valuation!E14)/1000,"0")&amp;"bn"</f>
+        <f>TEXT((Valuation!D10+Valuation!D16)/1000,"0")&amp;"-"&amp;TEXT((Valuation!E10+Valuation!E16)/1000,"0")&amp;"bn"</f>
         <v/>
       </c>
     </row>
@@ -849,24 +862,39 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>•  EBITDA is ESTIMATED (Abbott discloses segment margin, not EBITDA). Every figure's basis is on the Sources &amp; Methodology tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Tabs:  Summary  ·  Inputs &amp; Assumptions  ·  Nutrition Comps  ·  EPD Comps  ·  Valuation  ·  Sources &amp; Methodology</t>
+          <t>•  Carve-out adjustments applied: standalone/dis-synergy cost 1.5% (Nutrition) / 2.0% (EPD) of sales reduces EBITDA; an illustrative $1.5bn NEC risk deduction is netted off Nutrition EV. Both are editable on the Inputs tab [S20, S21]. Stranded costs sit at Abbott RemainCo, not the target [S22].</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>•  EBITDA is ESTIMATED (Abbott discloses segment margin, not EBITDA). Every figure's basis is on the Sources &amp; Methodology tab. See Sensitivity tab for the swing factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Indicative EV is post standalone/dis-synergy costs and (for Nutrition) post the illustrative NEC deduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Tabs:  Summary · Inputs &amp; Assumptions · Nutrition Comps · EPD Comps · Valuation · Sensitivity · Sources &amp; Methodology</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
@@ -880,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1056,98 +1084,183 @@
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>Selected multiple ranges (judgement — see rationale below)</t>
+          <t>Carve-out / standalone adjustments</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Multiple</t>
+          <t>Adjustment</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Nutrition low</t>
+          <t>Nutrition</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Nutrition high</t>
+          <t>EPD</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>EPD low</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>EPD high</t>
+          <t>Basis / source (see Sources tab)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Standalone cost / dis-synergy (% of sales)</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>ESTIMATE — corporate functions a standalone unit must rebuild; typical carve-out 1-3% of sales [S20]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Standalone-adjusted EBITDA ($m)</t>
+        </is>
+      </c>
+      <c r="B18" s="25">
+        <f>B12-B17*B8</f>
+        <v/>
+      </c>
+      <c r="C18" s="25">
+        <f>C12-C17*C8</f>
+        <v/>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>ESTIMATE = estimated EBITDA - standalone cost (drives EV/EBITDA). PE buyer bears this; a strategic may offset via synergies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>NEC litigation risk deduction ($m, applied to Nutrition EV)</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>ESTIMATE / ILLUSTRATIVE — buyer indemnity ask; not a booked Abbott provision. Verdicts $58-495m, many on appeal [S19, S21]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Selected multiple ranges (judgement — see rationale below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Nutrition low</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Nutrition high</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>EPD low</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>EPD high</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>EV / Sales</t>
         </is>
       </c>
-      <c r="B17" s="29" t="n">
+      <c r="B23" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="29" t="n">
+      <c r="C23" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D23" s="29" t="n">
         <v>2.5</v>
       </c>
-      <c r="E17" s="29" t="n">
+      <c r="E23" s="29" t="n">
         <v>3.5</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>EV / EBITDA</t>
         </is>
       </c>
-      <c r="B18" s="29" t="n">
+      <c r="B24" s="29" t="n">
         <v>11</v>
       </c>
-      <c r="C18" s="29" t="n">
+      <c r="C24" s="29" t="n">
         <v>15</v>
       </c>
-      <c r="D18" s="29" t="n">
+      <c r="D24" s="29" t="n">
         <v>11</v>
       </c>
-      <c r="E18" s="29" t="n">
+      <c r="E24" s="29" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Rationale for selected ranges</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>•  Nutrition: peak infant-formula comps (Reckitt/MJN 17.4x, Nestlé/Pfizer ~20-24x) DISCOUNTED for blended adult+pediatric mix and the NEC litigation overhang [S5].</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>•  EPD: premium end of branded-generics range (STADA 13.4x / 11.3x; Krka ~11.5x) given +9.2% growth and 23.7% margin; above mature Western generics (Hikma/Richter ~6x) [S6].</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>•  EBITDA is ESTIMATED — Abbott discloses segment operating margin, not segment EBITDA. Refine with carve-out quality-of-earnings financials [S4].</t>
         </is>
@@ -1156,10 +1269,10 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -1940,7 +2053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2007,15 +2120,15 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>EV / Sales</t>
+          <t>EV / Sales (reported sales)</t>
         </is>
       </c>
       <c r="B6" s="30">
-        <f>'Inputs &amp; Assumptions'!B17</f>
+        <f>'Inputs &amp; Assumptions'!B23</f>
         <v/>
       </c>
       <c r="C6" s="30">
-        <f>'Inputs &amp; Assumptions'!C17</f>
+        <f>'Inputs &amp; Assumptions'!C23</f>
         <v/>
       </c>
       <c r="D6" s="37">
@@ -2034,23 +2147,23 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>EV / EBITDA</t>
+          <t>EV / EBITDA (standalone EBITDA)</t>
         </is>
       </c>
       <c r="B7" s="30">
-        <f>'Inputs &amp; Assumptions'!B18</f>
+        <f>'Inputs &amp; Assumptions'!B24</f>
         <v/>
       </c>
       <c r="C7" s="30">
-        <f>'Inputs &amp; Assumptions'!C18</f>
+        <f>'Inputs &amp; Assumptions'!C24</f>
         <v/>
       </c>
       <c r="D7" s="37">
-        <f>'Inputs &amp; Assumptions'!B12*B7</f>
+        <f>'Inputs &amp; Assumptions'!B18*B7</f>
         <v/>
       </c>
       <c r="E7" s="37">
-        <f>'Inputs &amp; Assumptions'!B12*C7</f>
+        <f>'Inputs &amp; Assumptions'!B18*C7</f>
         <v/>
       </c>
       <c r="F7" s="38">
@@ -2061,7 +2174,7 @@
     <row r="8">
       <c r="A8" s="39" t="inlineStr">
         <is>
-          <t>Blended indicative EV</t>
+          <t>Blended indicative EV (pre-litigation)</t>
         </is>
       </c>
       <c r="B8" s="40" t="inlineStr"/>
@@ -2079,165 +2192,204 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>less: NEC litigation risk deduction</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr"/>
+      <c r="C9" s="20" t="inlineStr"/>
+      <c r="D9" s="37">
+        <f>-'Inputs &amp; Assumptions'!B19</f>
+        <v/>
+      </c>
+      <c r="E9" s="37">
+        <f>-'Inputs &amp; Assumptions'!B19</f>
+        <v/>
+      </c>
+      <c r="F9" s="20" t="inlineStr"/>
+    </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Adjusted indicative EV</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="inlineStr"/>
+      <c r="C10" s="27" t="inlineStr"/>
+      <c r="D10" s="25">
+        <f>D8-'Inputs &amp; Assumptions'!B19</f>
+        <v/>
+      </c>
+      <c r="E10" s="25">
+        <f>E8-'Inputs &amp; Assumptions'!B19</f>
+        <v/>
+      </c>
+      <c r="F10" s="43">
+        <f>AVERAGE(D10:E10)/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Established Pharmaceuticals (EPD)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Multiple low</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Multiple high</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>EV low ($m)</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>EV high ($m)</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>EV midpoint ($bn)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>EV / Sales</t>
-        </is>
-      </c>
-      <c r="B12" s="30">
-        <f>'Inputs &amp; Assumptions'!D17</f>
-        <v/>
-      </c>
-      <c r="C12" s="30">
-        <f>'Inputs &amp; Assumptions'!E17</f>
-        <v/>
-      </c>
-      <c r="D12" s="37">
-        <f>'Inputs &amp; Assumptions'!C8*B12</f>
-        <v/>
-      </c>
-      <c r="E12" s="37">
-        <f>'Inputs &amp; Assumptions'!C8*C12</f>
-        <v/>
-      </c>
-      <c r="F12" s="38">
-        <f>AVERAGE(D12:E12)/1000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>EV / EBITDA</t>
-        </is>
-      </c>
-      <c r="B13" s="30">
-        <f>'Inputs &amp; Assumptions'!D18</f>
-        <v/>
-      </c>
-      <c r="C13" s="30">
-        <f>'Inputs &amp; Assumptions'!E18</f>
-        <v/>
-      </c>
-      <c r="D13" s="37">
-        <f>'Inputs &amp; Assumptions'!C12*B13</f>
-        <v/>
-      </c>
-      <c r="E13" s="37">
-        <f>'Inputs &amp; Assumptions'!C12*C13</f>
-        <v/>
-      </c>
-      <c r="F13" s="38">
-        <f>AVERAGE(D13:E13)/1000</f>
-        <v/>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" s="39" t="inlineStr">
-        <is>
-          <t>Blended indicative EV</t>
-        </is>
-      </c>
-      <c r="B14" s="40" t="inlineStr"/>
-      <c r="C14" s="40" t="inlineStr"/>
-      <c r="D14" s="41">
-        <f>MIN(D12:E13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="41">
-        <f>MAX(D12:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="42">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>EV / Sales (reported sales)</t>
+        </is>
+      </c>
+      <c r="B14" s="30">
+        <f>'Inputs &amp; Assumptions'!D23</f>
+        <v/>
+      </c>
+      <c r="C14" s="30">
+        <f>'Inputs &amp; Assumptions'!E23</f>
+        <v/>
+      </c>
+      <c r="D14" s="37">
+        <f>'Inputs &amp; Assumptions'!C8*B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="37">
+        <f>'Inputs &amp; Assumptions'!C8*C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="38">
         <f>AVERAGE(D14:E14)/1000</f>
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>EV / EBITDA (standalone EBITDA)</t>
+        </is>
+      </c>
+      <c r="B15" s="30">
+        <f>'Inputs &amp; Assumptions'!D24</f>
+        <v/>
+      </c>
+      <c r="C15" s="30">
+        <f>'Inputs &amp; Assumptions'!E24</f>
+        <v/>
+      </c>
+      <c r="D15" s="37">
+        <f>'Inputs &amp; Assumptions'!C18*B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="37">
+        <f>'Inputs &amp; Assumptions'!C18*C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="38">
+        <f>AVERAGE(D15:E15)/1000</f>
+        <v/>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Combined (Nutrition + EPD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>Blended indicative EV (pre-litigation)</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="inlineStr"/>
+      <c r="C16" s="40" t="inlineStr"/>
+      <c r="D16" s="41">
+        <f>MIN(D14:E15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="41">
+        <f>MAX(D14:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="42">
+        <f>AVERAGE(D16:E16)/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Combined (Nutrition adjusted + EPD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>EV low ($m)</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>EV high ($m)</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>EV midpoint ($bn)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="24" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>Total indicative enterprise value</t>
         </is>
       </c>
-      <c r="B18" s="27" t="inlineStr"/>
-      <c r="C18" s="27" t="inlineStr"/>
-      <c r="D18" s="25">
-        <f>D8+D14</f>
-        <v/>
-      </c>
-      <c r="E18" s="25">
-        <f>E8+E14</f>
-        <v/>
-      </c>
-      <c r="F18" s="43">
-        <f>AVERAGE(D18:E18)/1000</f>
+      <c r="B21" s="27" t="inlineStr"/>
+      <c r="C21" s="27" t="inlineStr"/>
+      <c r="D21" s="25">
+        <f>D10+D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="25">
+        <f>E10+E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="43">
+        <f>AVERAGE(D21:E21)/1000</f>
         <v/>
       </c>
     </row>
@@ -2256,7 +2408,360 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Live grids driven by Inputs tab. Shows how indicative EV swings with the key carve-out estimates. $bn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>A.  Nutrition adjusted EV ($bn)  —  EV/EBITDA multiple  ×  standalone cost % of sales  (net of NEC deduction on Inputs tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>EV/EBITDA \ Std cost %</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C5" s="44" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D5" s="44" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E5" s="44" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="45" t="n">
+        <v>10</v>
+      </c>
+      <c r="B6" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*10/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="C6" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*10/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="D6" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*10/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="E6" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*10/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="B7" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*11/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="C7" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*11/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="D7" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*11/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="E7" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*11/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="45" t="n">
+        <v>12</v>
+      </c>
+      <c r="B8" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*12/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="C8" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*12/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="D8" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*12/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="E8" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*12/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="45" t="n">
+        <v>13</v>
+      </c>
+      <c r="B9" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*13/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="C9" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*13/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="D9" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*13/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="E9" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*13/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="45" t="n">
+        <v>14</v>
+      </c>
+      <c r="B10" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*14/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="C10" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*14/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="D10" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*14/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="E10" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*14/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*15/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="C11" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*15/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="D11" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*15/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+      <c r="E11" s="46">
+        <f>(('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*15/1000-'Inputs &amp; Assumptions'!B19/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>B.  Combined adjusted EV ($bn)  —  NEC deduction $bn (rows)  ×  standalone cost % applied to both (cols),  at selected EV/EBITDA midpoints</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>NEC $m \ Std cost %</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C14" s="44" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D14" s="44" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E14" s="44" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="B15" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-0+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.01*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="C15" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-0+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.015*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="D15" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-0+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.02*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="E15" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-0+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.025*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="47" t="n">
+        <v>500</v>
+      </c>
+      <c r="B16" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.01*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="C16" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.015*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="D16" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.02*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="E16" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.025*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="47" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B17" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.01*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="C17" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.015*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="D17" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.02*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="E17" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.025*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="47" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B18" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.01*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="C18" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.015*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="D18" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.02*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="E18" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-1500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.025*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="47" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B19" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.01*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="C19" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.015*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="D19" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.02*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="E19" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2000+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.025*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="47" t="n">
+        <v>2500</v>
+      </c>
+      <c r="B20" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.01*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.01*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="C20" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.015*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.015*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="D20" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.02*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.02*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+      <c r="E20" s="46">
+        <f>((('Inputs &amp; Assumptions'!B8*('Inputs &amp; Assumptions'!B9+'Inputs &amp; Assumptions'!B10))-0.025*'Inputs &amp; Assumptions'!B8)*((('Inputs &amp; Assumptions'!B24)+('Inputs &amp; Assumptions'!C24))/2)-2500+(('Inputs &amp; Assumptions'!C8*('Inputs &amp; Assumptions'!C9+'Inputs &amp; Assumptions'!C10))-0.025*'Inputs &amp; Assumptions'!C8)*((('Inputs &amp; Assumptions'!D24)+('Inputs &amp; Assumptions'!E24))/2))/1000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Tables use the EV/EBITDA method (the method affected by standalone costs); EV/Sales is unaffected. Shaded cells nearest the base case (1.5%/2.0% cost, $1.5bn NEC) are the headline. Estimates — not investment advice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2335,7 +2840,7 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E6" s="44" t="inlineStr">
+      <c r="E6" s="48" t="inlineStr">
         <is>
           <t>Abbott FY2024 Form 10-K (FY ended 31-Dec-2024)</t>
         </is>
@@ -2362,7 +2867,7 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E7" s="44" t="inlineStr">
+      <c r="E7" s="48" t="inlineStr">
         <is>
           <t>Abbott segment reporting (Bullfincher; Statista)</t>
         </is>
@@ -2389,7 +2894,7 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E8" s="44" t="inlineStr">
+      <c r="E8" s="48" t="inlineStr">
         <is>
           <t>Abbott FY2024 10-K MD&amp;A (segment results)</t>
         </is>
@@ -2411,12 +2916,12 @@
           <t>D&amp;A add-back 3.75% / 2.75%</t>
         </is>
       </c>
-      <c r="D9" s="45" t="inlineStr">
+      <c r="D9" s="49" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
       </c>
-      <c r="E9" s="44" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>Abbott FY2024 cash-flow disclosure (per 10-Q/10-K); segment split is analyst judgement</t>
         </is>
@@ -2438,7 +2943,7 @@
           <t>sales x margin</t>
         </is>
       </c>
-      <c r="D10" s="46" t="inlineStr">
+      <c r="D10" s="50" t="inlineStr">
         <is>
           <t>DERIVED</t>
         </is>
@@ -2465,7 +2970,7 @@
           <t>op earnings + D&amp;A</t>
         </is>
       </c>
-      <c r="D11" s="45" t="inlineStr">
+      <c r="D11" s="49" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
@@ -2526,7 +3031,7 @@
           <t>Peak comps discounted</t>
         </is>
       </c>
-      <c r="D15" s="45" t="inlineStr">
+      <c r="D15" s="49" t="inlineStr">
         <is>
           <t>ESTIMATE</t>
         </is>
@@ -2558,7 +3063,7 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E16" s="44" t="inlineStr">
+      <c r="E16" s="48" t="inlineStr">
         <is>
           <t>InterCapital — European pharma generics M&amp;A</t>
         </is>
@@ -2580,12 +3085,12 @@
           <t>€12.3bn EV; ~22x EBITDA; FY06 sales €2.6bn (18.4% EBITA margin)</t>
         </is>
       </c>
-      <c r="D17" s="46" t="inlineStr">
+      <c r="D17" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
       </c>
-      <c r="E17" s="44" t="inlineStr">
+      <c r="E17" s="48" t="inlineStr">
         <is>
           <t>Danone analyst presentation (Jul-2007); 22x cited in RB/MJN coverage</t>
         </is>
@@ -2607,12 +3112,12 @@
           <t>$5.5bn EV; 15.7x FY07e EBITDA; FY07e sales $1.95bn</t>
         </is>
       </c>
-      <c r="D18" s="46" t="inlineStr">
+      <c r="D18" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
       </c>
-      <c r="E18" s="44" t="inlineStr">
+      <c r="E18" s="48" t="inlineStr">
         <is>
           <t>Washington Post (Apr-2007); Nestlé/Novartis releases</t>
         </is>
@@ -2634,12 +3139,12 @@
           <t>$11.85bn EV; FY11 sales $2.1bn, EBITDA $0.5bn (=23.7x); press ~20x fwd</t>
         </is>
       </c>
-      <c r="D19" s="46" t="inlineStr">
+      <c r="D19" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
       </c>
-      <c r="E19" s="44" t="inlineStr">
+      <c r="E19" s="48" t="inlineStr">
         <is>
           <t>Proactive Investors; Pfizer 8-K (SEC)</t>
         </is>
@@ -2666,7 +3171,7 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E20" s="44" t="inlineStr">
+      <c r="E20" s="48" t="inlineStr">
         <is>
           <t>FoodNavigator-USA</t>
         </is>
@@ -2693,7 +3198,7 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E21" s="44" t="inlineStr">
+      <c r="E21" s="48" t="inlineStr">
         <is>
           <t>Bocconi BSIC; Mead Johnson 8-K (SEC)</t>
         </is>
@@ -2715,7 +3220,7 @@
           <t>$5.75bn EV; ~$2.0bn sales (=~2.9x); EBITDA n/d</t>
         </is>
       </c>
-      <c r="D22" s="46" t="inlineStr">
+      <c r="D22" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
@@ -2742,7 +3247,7 @@
           <t>~$4.0bn EV incl. debt; ~$1.8bn sales (=~2.2x); EBITDA n/d</t>
         </is>
       </c>
-      <c r="D23" s="46" t="inlineStr">
+      <c r="D23" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
@@ -2774,7 +3279,7 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E24" s="44" t="inlineStr">
+      <c r="E24" s="48" t="inlineStr">
         <is>
           <t>SEC Form 425 (Allergan); analyst commentary</t>
         </is>
@@ -2796,12 +3301,12 @@
           <t>$9.9bn EV; 8.9x adj. EBITDA w/ synergies; FY15 sales ~$2.3bn (=~4.0x)</t>
         </is>
       </c>
-      <c r="D25" s="46" t="inlineStr">
+      <c r="D25" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
       </c>
-      <c r="E25" s="44" t="inlineStr">
+      <c r="E25" s="48" t="inlineStr">
         <is>
           <t>Mylan 8-K (SEC)</t>
         </is>
@@ -2823,12 +3328,12 @@
           <t>€5.32bn EV; 13.4x FY16 EBITDA; FY16 sales €2.14bn (=~2.5x)</t>
         </is>
       </c>
-      <c r="D26" s="46" t="inlineStr">
+      <c r="D26" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
       </c>
-      <c r="E26" s="44" t="inlineStr">
+      <c r="E26" s="48" t="inlineStr">
         <is>
           <t>Bocconi BSIC</t>
         </is>
@@ -2850,12 +3355,12 @@
           <t>~€1.9bn EV; ~10.25x EBITDA; ~2.5x sales</t>
         </is>
       </c>
-      <c r="D27" s="46" t="inlineStr">
+      <c r="D27" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
       </c>
-      <c r="E27" s="44" t="inlineStr">
+      <c r="E27" s="48" t="inlineStr">
         <is>
           <t>InterCapital</t>
         </is>
@@ -2877,12 +3382,12 @@
           <t>~€10bn EV reported; ~11.29x EBITDA; FY24 sales ~€4.1bn (=~2.4x)</t>
         </is>
       </c>
-      <c r="D28" s="46" t="inlineStr">
+      <c r="D28" s="50" t="inlineStr">
         <is>
           <t>REPORTED/DERIVED</t>
         </is>
       </c>
-      <c r="E28" s="44" t="inlineStr">
+      <c r="E28" s="48" t="inlineStr">
         <is>
           <t>Bain Capital/Cinven press; InterCapital</t>
         </is>
@@ -2909,14 +3414,95 @@
           <t>REPORTED</t>
         </is>
       </c>
-      <c r="E29" s="44" t="inlineStr">
+      <c r="E29" s="48" t="inlineStr">
         <is>
           <t>Reuters/Yahoo; Top Class Actions</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="42" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>Standalone cost / dis-synergy assumption</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>1.5% (Nutrition) / 2.0% (EPD) of sales</t>
+        </is>
+      </c>
+      <c r="D30" s="49" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>Analyst judgement — typical carve-out dis-synergy 1-3% of revenue (corporate finance/IT/HR/legal/regulatory rebuilt; net of TSA). PE buyer bears; strategic may offset via synergies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>NEC litigation risk deduction (Nutrition EV)</t>
+        </is>
+      </c>
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>$1,500m (illustrative, editable)</t>
+        </is>
+      </c>
+      <c r="D31" s="49" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E31" s="20" t="inlineStr">
+        <is>
+          <t>Illustrative buyer indemnity/escrow ask — NOT a booked Abbott provision. Placeholder given unresolved litigation; Abbott has also won defense verdicts and is appealing [S19].</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Stranded costs at RemainCo (Abbott retained group)</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>Not deducted from target EV</t>
+        </is>
+      </c>
+      <c r="D32" s="49" t="inlineStr">
+        <is>
+          <t>ESTIMATE</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>Costs left behind that don't transfer with the unit affect Abbott's RemainCo, not the target's standalone EV; flagged for the seller's net-proceeds / dis-synergy analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Legend:  REPORTED = from a primary filing or press source  ·  DERIVED = calculated (EV ÷ sales/EBITDA)  ·  ESTIMATE = analyst judgement.  Multiples across sources may use different EBITDA definitions / years; treat as directional. Not investment advice.</t>
         </is>
@@ -2925,8 +3511,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A31:E31"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId1"/>

</xml_diff>